<commit_message>
hydrogen inventories without wind
</commit_message>
<xml_diff>
--- a/Plots/Prospective in Presmise tables.xlsx
+++ b/Plots/Prospective in Presmise tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20400"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10709"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Prospective LCA\Plots\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abhinabera/Desktop/Prospective-LCA/Plots/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F44409C0-5358-42E2-8469-7D3D57179108}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC3D1F8-7D8F-D041-A03D-27417E3D9621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13380" xr2:uid="{4D67D81B-D756-490A-95E0-BE3BCFD95BEB}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{4D67D81B-D756-490A-95E0-BE3BCFD95BEB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -129,9 +129,6 @@
     <t>No (optimised technology)</t>
   </si>
   <si>
-    <t>Yes (partial with only grid-based water electrolysis)</t>
-  </si>
-  <si>
     <r>
       <t>H</t>
     </r>
@@ -226,8 +223,17 @@
     <t>Main impacts</t>
   </si>
   <si>
-    <r>
-      <t>Yes (partial with only CO</t>
+    <t>Ethylene</t>
+  </si>
+  <si>
+    <t>green methanol to olefins</t>
+  </si>
+  <si>
+    <t>fossil methanol to olefins</t>
+  </si>
+  <si>
+    <r>
+      <t>Solar PV electricity + CO</t>
     </r>
     <r>
       <rPr>
@@ -246,67 +252,61 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve"> from DAC for methanol production</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Onshore wind electricity + CO</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> from DAC for methanol production</t>
+    </r>
+  </si>
+  <si>
+    <t>Yes (modeled with grid electricity)</t>
+  </si>
+  <si>
+    <t>Yes (modeled with only grid-based water electrolysis)</t>
+  </si>
+  <si>
+    <r>
+      <t>Yes (with only CO</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve"> from DAC)</t>
-    </r>
-  </si>
-  <si>
-    <t>Yes (partial with grid electricity)</t>
-  </si>
-  <si>
-    <t>Ethylene</t>
-  </si>
-  <si>
-    <t>green methanol to olefins</t>
-  </si>
-  <si>
-    <t>fossil methanol to olefins</t>
-  </si>
-  <si>
-    <r>
-      <t>Solar PV electricity + CO</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> from DAC for methanol production</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Onshore wind electricity + CO</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> from DAC for methanol production</t>
     </r>
   </si>
 </sst>
@@ -374,7 +374,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -397,11 +397,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -438,6 +464,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -762,18 +794,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0FCE10C-FBB8-4260-9A0D-EEF288A16D27}">
   <dimension ref="B2:F24"/>
-  <sheetFormatPr defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="11" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="5.77734375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" style="1"/>
+    <col min="2" max="2" width="5.83203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="16.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="1"/>
+    <col min="6" max="6" width="12.5" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" ht="12" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:6" ht="12" x14ac:dyDescent="0.15">
       <c r="B2" s="12" t="s">
         <v>0</v>
       </c>
@@ -782,7 +814,7 @@
       <c r="E2" s="12"/>
       <c r="F2" s="12"/>
     </row>
-    <row r="3" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:6" ht="24" x14ac:dyDescent="0.15">
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
@@ -793,13 +825,13 @@
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:6" ht="24" x14ac:dyDescent="0.15">
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
@@ -816,15 +848,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:6" ht="36.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>26</v>
+      <c r="D5" s="14" t="s">
+        <v>29</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>10</v>
@@ -833,12 +865,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="2:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:6" ht="36.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="10"/>
-      <c r="D6" s="11"/>
+      <c r="D6" s="15"/>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
@@ -846,7 +878,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:6" ht="12" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:6" ht="12" x14ac:dyDescent="0.15">
       <c r="B8" s="12" t="s">
         <v>13</v>
       </c>
@@ -855,7 +887,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
     </row>
-    <row r="9" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:6" ht="24" x14ac:dyDescent="0.15">
       <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
@@ -866,13 +898,13 @@
         <v>2</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:6" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:6" ht="40.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
@@ -889,7 +921,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="2:6" ht="35.4" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:6" ht="35.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="2" t="s">
         <v>4</v>
       </c>
@@ -897,7 +929,7 @@
         <v>16</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>10</v>
@@ -906,7 +938,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:6" ht="35.4" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:6" ht="35.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B12" s="2" t="s">
         <v>5</v>
       </c>
@@ -919,7 +951,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:6" ht="12" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:6" ht="12" x14ac:dyDescent="0.15">
       <c r="B14" s="12" t="s">
         <v>17</v>
       </c>
@@ -928,7 +960,7 @@
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
     </row>
-    <row r="15" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:6" ht="24" x14ac:dyDescent="0.15">
       <c r="B15" s="2" t="s">
         <v>7</v>
       </c>
@@ -939,13 +971,13 @@
         <v>2</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="2:6" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:6" ht="40.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B16" s="2" t="s">
         <v>3</v>
       </c>
@@ -962,46 +994,46 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B17" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>22</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:6" ht="36" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B18" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="11"/>
       <c r="E18" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" ht="12" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" ht="12" x14ac:dyDescent="0.15">
       <c r="B20" s="12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
     </row>
-    <row r="21" spans="2:6" ht="20.399999999999999" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:6" ht="24" x14ac:dyDescent="0.15">
       <c r="B21" s="2" t="s">
         <v>7</v>
       </c>
@@ -1012,18 +1044,18 @@
         <v>2</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F21" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="2:6" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:6" ht="40.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B22" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>12</v>
@@ -1035,38 +1067,43 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="2:6" ht="38.4" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:6" ht="38.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B23" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="2:6" ht="38.4" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:6" ht="38.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B24" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="13"/>
       <c r="E24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="9" t="s">
         <v>31</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
     <mergeCell ref="C11:C12"/>
     <mergeCell ref="D11:D12"/>
     <mergeCell ref="B14:F14"/>
@@ -1074,11 +1111,6 @@
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>